<commit_message>
feat: Xccelera AI generated project
</commit_message>
<xml_diff>
--- a/api_test_report.xlsx
+++ b/api_test_report.xlsx
@@ -882,21 +882,21 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>/api/v1/integrations/{id}</t>
+          <t>/api/v1/repositories</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Delete integration</t>
+          <t>Create repository</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
@@ -911,21 +911,21 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>/api/v1/repositories</t>
+          <t>/api/v1/repositories/{id}</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Create repository</t>
+          <t>Get repository</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
@@ -940,7 +940,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PUT</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -950,7 +950,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Get repository</t>
+          <t>Update repository</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
@@ -969,21 +969,21 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>PUT</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>/api/v1/repositories/{id}</t>
+          <t>/api/v1/deployments</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Update repository</t>
+          <t>Create deployment</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
@@ -998,21 +998,21 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>/api/v1/deployments</t>
+          <t>/api/v1/deployments/{id}</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Create deployment</t>
+          <t>Get deployment</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>

</xml_diff>